<commit_message>
HPE Bid (XLSX): flatten line numbering to a single 1..N sequence
BundleDetails rows are no longer sub-numbered under their parent bundle
(1.01, 1.02, ...); every emitted line now takes the next number in one
running sequence. Comment placement is unchanged (Max Qty only on Bundle/
Part Number lines). Updated File1 tests, regenerated its goldens, and
refreshed the HPE format spec + output mapping docs.
</commit_message>
<xml_diff>
--- a/samples/outputs/HPE_Deal_1601962887_v2_NoCalculation_parsed.xlsx
+++ b/samples/outputs/HPE_Deal_1601962887_v2_NoCalculation_parsed.xlsx
@@ -117,7 +117,7 @@
     <x:t>Max Qty: 1</x:t>
   </x:si>
   <x:si>
-    <x:t>1.01</x:t>
+    <x:t>2</x:t>
   </x:si>
   <x:si>
     <x:t>AK379B</x:t>
@@ -126,7 +126,7 @@
     <x:t>HPE MSL2024 Gen4 0-drive 24-slot Lib</x:t>
   </x:si>
   <x:si>
-    <x:t>1.02</x:t>
+    <x:t>3</x:t>
   </x:si>
   <x:si>
     <x:t>R6Q75A</x:t>
@@ -135,7 +135,7 @@
     <x:t>HPE MSL LTO-9 45000 SAS Drv Upg Kit</x:t>
   </x:si>
   <x:si>
-    <x:t>1.03</x:t>
+    <x:t>4</x:t>
   </x:si>
   <x:si>
     <x:t>TC406AAE</x:t>
@@ -144,7 +144,7 @@
     <x:t>HPE MSL CVTL-TapeAssure Adv E-LTU</x:t>
   </x:si>
   <x:si>
-    <x:t>1.04</x:t>
+    <x:t>5</x:t>
   </x:si>
   <x:si>
     <x:t>716191-B21</x:t>
@@ -153,7 +153,7 @@
     <x:t>HPE Ext 2.0m MiniSAS HD to MiniSAS Cbl</x:t>
   </x:si>
   <x:si>
-    <x:t>1.05</x:t>
+    <x:t>6</x:t>
   </x:si>
   <x:si>
     <x:t>C7978A</x:t>
@@ -162,7 +162,7 @@
     <x:t>HPE Ultrium Universal Cleaning Cartridge</x:t>
   </x:si>
   <x:si>
-    <x:t>1.06</x:t>
+    <x:t>7</x:t>
   </x:si>
   <x:si>
     <x:t>Q2079AN</x:t>
@@ -171,7 +171,7 @@
     <x:t>HPE LTO-9 45TB RW Non Cust Lbl 20 Crtg</x:t>
   </x:si>
   <x:si>
-    <x:t>1.07</x:t>
+    <x:t>8</x:t>
   </x:si>
   <x:si>
     <x:t>HU4B2A3</x:t>
@@ -180,19 +180,19 @@
     <x:t>HPE 3Y Tech Care Basic SVC</x:t>
   </x:si>
   <x:si>
-    <x:t>1.08</x:t>
+    <x:t>9</x:t>
   </x:si>
   <x:si>
     <x:t>HPE MSL TapeAssure Adv Lic Support</x:t>
   </x:si>
   <x:si>
-    <x:t>1.09</x:t>
+    <x:t>10</x:t>
   </x:si>
   <x:si>
     <x:t>HPE MSL2024 Library Support</x:t>
   </x:si>
   <x:si>
-    <x:t>2</x:t>
+    <x:t>11</x:t>
   </x:si>
   <x:si>
     <x:t>52079278</x:t>
@@ -201,7 +201,7 @@
     <x:t>Storeonce 80TB</x:t>
   </x:si>
   <x:si>
-    <x:t>2.01</x:t>
+    <x:t>12</x:t>
   </x:si>
   <x:si>
     <x:t>R6U02A</x:t>
@@ -210,7 +210,7 @@
     <x:t>HPE StoreOnce 3660 80TB Base System</x:t>
   </x:si>
   <x:si>
-    <x:t>2.02</x:t>
+    <x:t>13</x:t>
   </x:si>
   <x:si>
     <x:t>R7M24A</x:t>
@@ -219,13 +219,13 @@
     <x:t>HPE StoreOnce Gen4+ 10/25Gb 2p SFP Adptr</x:t>
   </x:si>
   <x:si>
-    <x:t>2.03</x:t>
+    <x:t>14</x:t>
   </x:si>
   <x:si>
     <x:t>Factory Integrated</x:t>
   </x:si>
   <x:si>
-    <x:t>2.04</x:t>
+    <x:t>15</x:t>
   </x:si>
   <x:si>
     <x:t>BB983A</x:t>
@@ -234,13 +234,13 @@
     <x:t>HPE StoreOnce Gen4 10/25Gb SFP Card LTU</x:t>
   </x:si>
   <x:si>
-    <x:t>2.05</x:t>
+    <x:t>16</x:t>
   </x:si>
   <x:si>
     <x:t>FACTORY INTEGRATED</x:t>
   </x:si>
   <x:si>
-    <x:t>2.06</x:t>
+    <x:t>17</x:t>
   </x:si>
   <x:si>
     <x:t>BB994AAE</x:t>
@@ -249,7 +249,7 @@
     <x:t>HPE StoreOnce Encryption E-LTU</x:t>
   </x:si>
   <x:si>
-    <x:t>2.07</x:t>
+    <x:t>18</x:t>
   </x:si>
   <x:si>
     <x:t>HU4A6A3</x:t>
@@ -258,13 +258,13 @@
     <x:t>HPE 3Y Tech Care Essential SVC</x:t>
   </x:si>
   <x:si>
-    <x:t>2.08</x:t>
+    <x:t>19</x:t>
   </x:si>
   <x:si>
     <x:t>HPE StoreOnce 3660 80TB Base System Supp</x:t>
   </x:si>
   <x:si>
-    <x:t>2.09</x:t>
+    <x:t>20</x:t>
   </x:si>
   <x:si>
     <x:t>HA124A1</x:t>
@@ -273,13 +273,13 @@
     <x:t>HPE Technical Installation Startup SVC</x:t>
   </x:si>
   <x:si>
-    <x:t>2.10</x:t>
+    <x:t>21</x:t>
   </x:si>
   <x:si>
     <x:t>HPE StoreOnce 36xx Stup SVC</x:t>
   </x:si>
   <x:si>
-    <x:t>2.11</x:t>
+    <x:t>22</x:t>
   </x:si>
   <x:si>
     <x:t>H33XYA1</x:t>
@@ -288,7 +288,7 @@
     <x:t>HPE Learn Credits for Storage SVC</x:t>
   </x:si>
   <x:si>
-    <x:t>3</x:t>
+    <x:t>23</x:t>
   </x:si>
   <x:si>
     <x:t>52079277</x:t>
@@ -297,7 +297,7 @@
     <x:t>Backup server</x:t>
   </x:si>
   <x:si>
-    <x:t>3.01</x:t>
+    <x:t>24</x:t>
   </x:si>
   <x:si>
     <x:t>P52499-B21</x:t>
@@ -306,10 +306,10 @@
     <x:t>HPE DL360 Gen11 8SFF CTO Server</x:t>
   </x:si>
   <x:si>
-    <x:t>3.02</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3.03</x:t>
+    <x:t>25</x:t>
+  </x:si>
+  <x:si>
+    <x:t>26</x:t>
   </x:si>
   <x:si>
     <x:t>P67079-B21</x:t>
@@ -318,13 +318,13 @@
     <x:t>INT Xeon-G 5515+ CPU for HPE</x:t>
   </x:si>
   <x:si>
-    <x:t>3.04</x:t>
+    <x:t>27</x:t>
   </x:si>
   <x:si>
     <x:t>Factory integrated</x:t>
   </x:si>
   <x:si>
-    <x:t>3.05</x:t>
+    <x:t>28</x:t>
   </x:si>
   <x:si>
     <x:t>P64706-B21</x:t>
@@ -333,10 +333,10 @@
     <x:t>HPE 32GB 2Rx8 PC5-5600B-R Smart Kit</x:t>
   </x:si>
   <x:si>
-    <x:t>3.06</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3.07</x:t>
+    <x:t>29</x:t>
+  </x:si>
+  <x:si>
+    <x:t>30</x:t>
   </x:si>
   <x:si>
     <x:t>P48895-B21</x:t>
@@ -345,10 +345,10 @@
     <x:t>HPE DL360 G11 8SFF x1 U.3 TM BP Kit</x:t>
   </x:si>
   <x:si>
-    <x:t>3.08</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3.09</x:t>
+    <x:t>31</x:t>
+  </x:si>
+  <x:si>
+    <x:t>32</x:t>
   </x:si>
   <x:si>
     <x:t>804398-B21</x:t>
@@ -357,10 +357,10 @@
     <x:t>HPE Smart Array E208e-p SR Gen10 Ctrlr</x:t>
   </x:si>
   <x:si>
-    <x:t>3.10</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3.11</x:t>
+    <x:t>33</x:t>
+  </x:si>
+  <x:si>
+    <x:t>34</x:t>
   </x:si>
   <x:si>
     <x:t>P26259-B21</x:t>
@@ -369,10 +369,10 @@
     <x:t>BCM 57412 10GbE 2p SFP+ Adptr</x:t>
   </x:si>
   <x:si>
-    <x:t>3.12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3.13</x:t>
+    <x:t>35</x:t>
+  </x:si>
+  <x:si>
+    <x:t>36</x:t>
   </x:si>
   <x:si>
     <x:t>P01366-B21</x:t>
@@ -381,10 +381,10 @@
     <x:t>HPE 96W Smart Stg Li-ion Batt 145mm Kit</x:t>
   </x:si>
   <x:si>
-    <x:t>3.14</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3.15</x:t>
+    <x:t>37</x:t>
+  </x:si>
+  <x:si>
+    <x:t>38</x:t>
   </x:si>
   <x:si>
     <x:t>P48918-B21</x:t>
@@ -393,10 +393,10 @@
     <x:t>HPE DL360 Gen11 Stg Cntrl Enable Cbl Kit</x:t>
   </x:si>
   <x:si>
-    <x:t>3.16</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3.17</x:t>
+    <x:t>39</x:t>
+  </x:si>
+  <x:si>
+    <x:t>40</x:t>
   </x:si>
   <x:si>
     <x:t>P58335-B21</x:t>
@@ -405,10 +405,10 @@
     <x:t>HPE MR408i-o Gen11 SPDM Storage Cntlr</x:t>
   </x:si>
   <x:si>
-    <x:t>3.18</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3.19</x:t>
+    <x:t>41</x:t>
+  </x:si>
+  <x:si>
+    <x:t>42</x:t>
   </x:si>
   <x:si>
     <x:t>P51181-B21</x:t>
@@ -417,10 +417,10 @@
     <x:t>BCM 5719 1Gb 4p BASE-T OCP Adptr</x:t>
   </x:si>
   <x:si>
-    <x:t>3.20</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3.21</x:t>
+    <x:t>43</x:t>
+  </x:si>
+  <x:si>
+    <x:t>44</x:t>
   </x:si>
   <x:si>
     <x:t>P48908-B21</x:t>
@@ -429,10 +429,10 @@
     <x:t>HPE DL3X0 Gen11 1U High Perf Fan Kit</x:t>
   </x:si>
   <x:si>
-    <x:t>3.22</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3.23</x:t>
+    <x:t>45</x:t>
+  </x:si>
+  <x:si>
+    <x:t>46</x:t>
   </x:si>
   <x:si>
     <x:t>P38995-B21</x:t>
@@ -441,10 +441,10 @@
     <x:t>HPE 800W FS Plat Ht Plg LH Pwr Sply Kit</x:t>
   </x:si>
   <x:si>
-    <x:t>3.24</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3.25</x:t>
+    <x:t>47</x:t>
+  </x:si>
+  <x:si>
+    <x:t>48</x:t>
   </x:si>
   <x:si>
     <x:t>BD505A</x:t>
@@ -453,10 +453,10 @@
     <x:t>HPE iLO Adv 1-svr Lic 3yr Support</x:t>
   </x:si>
   <x:si>
-    <x:t>3.26</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3.27</x:t>
+    <x:t>49</x:t>
+  </x:si>
+  <x:si>
+    <x:t>50</x:t>
   </x:si>
   <x:si>
     <x:t>S1A05A</x:t>
@@ -465,7 +465,7 @@
     <x:t>HPE Cmp Cloud Mgmt Srv FIO Enablement</x:t>
   </x:si>
   <x:si>
-    <x:t>3.28</x:t>
+    <x:t>51</x:t>
   </x:si>
   <x:si>
     <x:t>P51911-B21</x:t>
@@ -474,10 +474,10 @@
     <x:t>HPE DL360 Gen11 CPU1/OCP2 x8 Enable Kit</x:t>
   </x:si>
   <x:si>
-    <x:t>3.29</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3.30</x:t>
+    <x:t>52</x:t>
+  </x:si>
+  <x:si>
+    <x:t>53</x:t>
   </x:si>
   <x:si>
     <x:t>P52416-B21</x:t>
@@ -486,10 +486,10 @@
     <x:t>HPE DL360 Gen11 OROC TM Cbl Kit</x:t>
   </x:si>
   <x:si>
-    <x:t>3.31</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3.32</x:t>
+    <x:t>54</x:t>
+  </x:si>
+  <x:si>
+    <x:t>55</x:t>
   </x:si>
   <x:si>
     <x:t>P35876-B21</x:t>
@@ -498,7 +498,7 @@
     <x:t>HPE CE Mark Removal FIO Enable Kit</x:t>
   </x:si>
   <x:si>
-    <x:t>3.33</x:t>
+    <x:t>56</x:t>
   </x:si>
   <x:si>
     <x:t>P48183-B21</x:t>
@@ -507,10 +507,10 @@
     <x:t>HPE NS204i-u Gen11 Ht Plg Boot Opt Dev</x:t>
   </x:si>
   <x:si>
-    <x:t>3.34</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3.35</x:t>
+    <x:t>57</x:t>
+  </x:si>
+  <x:si>
+    <x:t>58</x:t>
   </x:si>
   <x:si>
     <x:t>P48905-B21</x:t>
@@ -519,10 +519,10 @@
     <x:t>HPE DL360 Gen11 High Perf Heat Sink Kit</x:t>
   </x:si>
   <x:si>
-    <x:t>3.36</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3.37</x:t>
+    <x:t>59</x:t>
+  </x:si>
+  <x:si>
+    <x:t>60</x:t>
   </x:si>
   <x:si>
     <x:t>P48920-B21</x:t>
@@ -531,10 +531,10 @@
     <x:t>HPE DL360 Gen11 NS204i-u Front Cbl Kit</x:t>
   </x:si>
   <x:si>
-    <x:t>3.38</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3.39</x:t>
+    <x:t>61</x:t>
+  </x:si>
+  <x:si>
+    <x:t>62</x:t>
   </x:si>
   <x:si>
     <x:t>P52341-B21</x:t>
@@ -543,10 +543,10 @@
     <x:t>HPE DL3XX Gen11 Easy Install Rail 3 Kit</x:t>
   </x:si>
   <x:si>
-    <x:t>3.40</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3.41</x:t>
+    <x:t>63</x:t>
+  </x:si>
+  <x:si>
+    <x:t>64</x:t>
   </x:si>
   <x:si>
     <x:t>R7A11AAE</x:t>
@@ -555,10 +555,10 @@
     <x:t>HPE COM Std 3yr Up ProLiant SaaS</x:t>
   </x:si>
   <x:si>
-    <x:t>3.42</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3.43</x:t>
+    <x:t>65</x:t>
+  </x:si>
+  <x:si>
+    <x:t>66</x:t>
   </x:si>
   <x:si>
     <x:t>HU4A6A300DJ</x:t>

</xml_diff>